<commit_message>
Slightly less thread unsafe
</commit_message>
<xml_diff>
--- a/Output/output_test.xlsx
+++ b/Output/output_test.xlsx
@@ -97,15 +97,48 @@
     <t>VIVID - 1</t>
   </si>
   <si>
+    <t>VIVID - 2</t>
+  </si>
+  <si>
+    <t>VIVID - 3</t>
+  </si>
+  <si>
     <t>VIVID - 4</t>
   </si>
   <si>
+    <t>VIVID - 5</t>
+  </si>
+  <si>
     <t>VIVID - 6</t>
   </si>
   <si>
+    <t>VIVID - 7</t>
+  </si>
+  <si>
+    <t>VIVID - 8</t>
+  </si>
+  <si>
+    <t>VIVID - 9</t>
+  </si>
+  <si>
     <t>VIVID - 10</t>
   </si>
   <si>
+    <t>VIVID - 11</t>
+  </si>
+  <si>
+    <t>VIVID - 12</t>
+  </si>
+  <si>
+    <t>VIVID - 13</t>
+  </si>
+  <si>
+    <t>VIVID - 14</t>
+  </si>
+  <si>
+    <t>VIVID - 15</t>
+  </si>
+  <si>
     <t>VIVID - 16</t>
   </si>
   <si>
@@ -115,40 +148,7 @@
     <t>VIVID - 18</t>
   </si>
   <si>
-    <t>VIVID - 20</t>
-  </si>
-  <si>
-    <t>VIVID - 21</t>
-  </si>
-  <si>
-    <t>VIVID - 22</t>
-  </si>
-  <si>
-    <t>VIVID - 24</t>
-  </si>
-  <si>
-    <t>VIVID - 25</t>
-  </si>
-  <si>
-    <t>VIVID - 27</t>
-  </si>
-  <si>
-    <t>VIVID - 32</t>
-  </si>
-  <si>
-    <t>VIVID - 34</t>
-  </si>
-  <si>
-    <t>VIVID - 37</t>
-  </si>
-  <si>
-    <t>VIVID - 43</t>
-  </si>
-  <si>
-    <t>VIVID - 44</t>
-  </si>
-  <si>
-    <t>VIVID - 48</t>
+    <t>VIVID - 19</t>
   </si>
   <si>
     <t>Baltimore Orioles vs Toronto Blue Jays [4/25/2012] Tickets at StubHub!</t>
@@ -660,7 +660,7 @@
         <v>65</v>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -677,7 +677,7 @@
         <v>66</v>
       </c>
       <c r="E3">
-        <v>74.07407407407408</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -694,7 +694,7 @@
         <v>67</v>
       </c>
       <c r="E4">
-        <v>68.9655172413793</v>
+        <v>31.48148148148148</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -711,7 +711,7 @@
         <v>68</v>
       </c>
       <c r="E5">
-        <v>71.42857142857143</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -728,7 +728,7 @@
         <v>69</v>
       </c>
       <c r="E6">
-        <v>70.17543859649123</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -745,7 +745,7 @@
         <v>70</v>
       </c>
       <c r="E7">
-        <v>31.48148148148148</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -762,7 +762,7 @@
         <v>71</v>
       </c>
       <c r="E8">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -779,7 +779,7 @@
         <v>72</v>
       </c>
       <c r="E9">
-        <v>33.64485981308411</v>
+        <v>28.0373831775701</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -796,7 +796,7 @@
         <v>73</v>
       </c>
       <c r="E10">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -813,7 +813,7 @@
         <v>74</v>
       </c>
       <c r="E11">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -830,7 +830,7 @@
         <v>75</v>
       </c>
       <c r="E12">
-        <v>29.41176470588235</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -847,7 +847,7 @@
         <v>76</v>
       </c>
       <c r="E13">
-        <v>31.06796116504854</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -864,7 +864,7 @@
         <v>77</v>
       </c>
       <c r="E14">
-        <v>28.28282828282828</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -881,7 +881,7 @@
         <v>78</v>
       </c>
       <c r="E15">
-        <v>33.00970873786407</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -898,7 +898,7 @@
         <v>79</v>
       </c>
       <c r="E16">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -915,7 +915,7 @@
         <v>80</v>
       </c>
       <c r="E17">
-        <v>74.07407407407408</v>
+        <v>42.30769230769231</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -932,7 +932,7 @@
         <v>81</v>
       </c>
       <c r="E18">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -949,7 +949,7 @@
         <v>82</v>
       </c>
       <c r="E19">
-        <v>31.77570093457943</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -966,7 +966,7 @@
         <v>83</v>
       </c>
       <c r="E20">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -983,7 +983,7 @@
         <v>84</v>
       </c>
       <c r="E21">
-        <v>31.68316831683168</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1000,7 +1000,7 @@
         <v>65</v>
       </c>
       <c r="E22">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1017,7 +1017,7 @@
         <v>65</v>
       </c>
       <c r="E23">
-        <v>68.9655172413793</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1034,7 +1034,7 @@
         <v>66</v>
       </c>
       <c r="E24">
-        <v>100</v>
+        <v>38.38383838383839</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1051,7 +1051,7 @@
         <v>67</v>
       </c>
       <c r="E25">
-        <v>68.9655172413793</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1068,7 +1068,7 @@
         <v>68</v>
       </c>
       <c r="E26">
-        <v>71.42857142857143</v>
+        <v>33.66336633663366</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1085,7 +1085,7 @@
         <v>69</v>
       </c>
       <c r="E27">
-        <v>70.17543859649123</v>
+        <v>33.33333333333334</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1102,7 +1102,7 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>33.00970873786407</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1119,7 +1119,7 @@
         <v>71</v>
       </c>
       <c r="E29">
-        <v>31.57894736842105</v>
+        <v>27.36842105263158</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1136,7 +1136,7 @@
         <v>72</v>
       </c>
       <c r="E30">
-        <v>33.33333333333333</v>
+        <v>31.37254901960784</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -1153,7 +1153,7 @@
         <v>73</v>
       </c>
       <c r="E31">
-        <v>31.25</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -1170,7 +1170,7 @@
         <v>74</v>
       </c>
       <c r="E32">
-        <v>33.33333333333333</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -1187,7 +1187,7 @@
         <v>75</v>
       </c>
       <c r="E33">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -1204,7 +1204,7 @@
         <v>76</v>
       </c>
       <c r="E34">
-        <v>32.65306122448979</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -1221,7 +1221,7 @@
         <v>77</v>
       </c>
       <c r="E35">
-        <v>29.78723404255319</v>
+        <v>25.53191489361702</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1238,7 +1238,7 @@
         <v>78</v>
       </c>
       <c r="E36">
-        <v>36.73469387755102</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -1255,7 +1255,7 @@
         <v>79</v>
       </c>
       <c r="E37">
-        <v>35.64356435643565</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -1272,7 +1272,7 @@
         <v>80</v>
       </c>
       <c r="E38">
-        <v>34.34343434343434</v>
+        <v>28.28282828282829</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -1289,7 +1289,7 @@
         <v>81</v>
       </c>
       <c r="E39">
-        <v>33.33333333333333</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1306,7 +1306,7 @@
         <v>82</v>
       </c>
       <c r="E40">
-        <v>31.37254901960785</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1323,7 +1323,7 @@
         <v>83</v>
       </c>
       <c r="E41">
-        <v>31.68316831683168</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -1340,7 +1340,7 @@
         <v>84</v>
       </c>
       <c r="E42">
-        <v>33.33333333333333</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -1357,7 +1357,7 @@
         <v>66</v>
       </c>
       <c r="E43">
-        <v>100</v>
+        <v>38.38383838383839</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -1374,7 +1374,7 @@
         <v>65</v>
       </c>
       <c r="E44">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -1391,7 +1391,7 @@
         <v>66</v>
       </c>
       <c r="E45">
-        <v>74.07407407407408</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -1408,7 +1408,7 @@
         <v>67</v>
       </c>
       <c r="E46">
-        <v>68.9655172413793</v>
+        <v>31.48148148148148</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -1425,7 +1425,7 @@
         <v>68</v>
       </c>
       <c r="E47">
-        <v>71.42857142857143</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -1442,7 +1442,7 @@
         <v>69</v>
       </c>
       <c r="E48">
-        <v>70.17543859649123</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -1459,7 +1459,7 @@
         <v>70</v>
       </c>
       <c r="E49">
-        <v>31.48148148148148</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -1476,7 +1476,7 @@
         <v>71</v>
       </c>
       <c r="E50">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -1493,7 +1493,7 @@
         <v>72</v>
       </c>
       <c r="E51">
-        <v>33.64485981308411</v>
+        <v>28.0373831775701</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -1510,7 +1510,7 @@
         <v>73</v>
       </c>
       <c r="E52">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -1527,7 +1527,7 @@
         <v>74</v>
       </c>
       <c r="E53">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -1544,7 +1544,7 @@
         <v>75</v>
       </c>
       <c r="E54">
-        <v>29.41176470588235</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -1561,7 +1561,7 @@
         <v>76</v>
       </c>
       <c r="E55">
-        <v>31.06796116504854</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -1578,7 +1578,7 @@
         <v>77</v>
       </c>
       <c r="E56">
-        <v>28.28282828282828</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -1595,7 +1595,7 @@
         <v>78</v>
       </c>
       <c r="E57">
-        <v>33.00970873786407</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -1612,7 +1612,7 @@
         <v>79</v>
       </c>
       <c r="E58">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -1629,7 +1629,7 @@
         <v>80</v>
       </c>
       <c r="E59">
-        <v>74.07407407407408</v>
+        <v>42.30769230769231</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -1646,7 +1646,7 @@
         <v>81</v>
       </c>
       <c r="E60">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -1663,7 +1663,7 @@
         <v>82</v>
       </c>
       <c r="E61">
-        <v>31.77570093457943</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -1680,7 +1680,7 @@
         <v>83</v>
       </c>
       <c r="E62">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -1697,7 +1697,7 @@
         <v>84</v>
       </c>
       <c r="E63">
-        <v>31.68316831683168</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -1714,7 +1714,7 @@
         <v>65</v>
       </c>
       <c r="E64">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -1731,7 +1731,7 @@
         <v>65</v>
       </c>
       <c r="E65">
-        <v>68.9655172413793</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -1748,7 +1748,7 @@
         <v>66</v>
       </c>
       <c r="E66">
-        <v>100</v>
+        <v>38.38383838383839</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -1765,7 +1765,7 @@
         <v>67</v>
       </c>
       <c r="E67">
-        <v>68.9655172413793</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -1782,7 +1782,7 @@
         <v>68</v>
       </c>
       <c r="E68">
-        <v>71.42857142857143</v>
+        <v>33.66336633663366</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -1799,7 +1799,7 @@
         <v>69</v>
       </c>
       <c r="E69">
-        <v>70.17543859649123</v>
+        <v>33.33333333333334</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -1816,7 +1816,7 @@
         <v>70</v>
       </c>
       <c r="E70">
-        <v>33.00970873786407</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -1833,7 +1833,7 @@
         <v>71</v>
       </c>
       <c r="E71">
-        <v>31.57894736842105</v>
+        <v>27.36842105263158</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -1850,7 +1850,7 @@
         <v>72</v>
       </c>
       <c r="E72">
-        <v>33.33333333333333</v>
+        <v>31.37254901960784</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -1867,7 +1867,7 @@
         <v>73</v>
       </c>
       <c r="E73">
-        <v>31.25</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -1884,7 +1884,7 @@
         <v>74</v>
       </c>
       <c r="E74">
-        <v>33.33333333333333</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -1901,7 +1901,7 @@
         <v>75</v>
       </c>
       <c r="E75">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -1918,7 +1918,7 @@
         <v>76</v>
       </c>
       <c r="E76">
-        <v>32.65306122448979</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -1935,7 +1935,7 @@
         <v>77</v>
       </c>
       <c r="E77">
-        <v>29.78723404255319</v>
+        <v>25.53191489361702</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -1952,7 +1952,7 @@
         <v>78</v>
       </c>
       <c r="E78">
-        <v>36.73469387755102</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -1969,7 +1969,7 @@
         <v>79</v>
       </c>
       <c r="E79">
-        <v>35.64356435643565</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -1986,7 +1986,7 @@
         <v>80</v>
       </c>
       <c r="E80">
-        <v>34.34343434343434</v>
+        <v>28.28282828282829</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -2003,7 +2003,7 @@
         <v>81</v>
       </c>
       <c r="E81">
-        <v>33.33333333333333</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -2020,7 +2020,7 @@
         <v>82</v>
       </c>
       <c r="E82">
-        <v>31.37254901960785</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -2037,7 +2037,7 @@
         <v>83</v>
       </c>
       <c r="E83">
-        <v>31.68316831683168</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -2054,7 +2054,7 @@
         <v>84</v>
       </c>
       <c r="E84">
-        <v>33.33333333333333</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -2071,7 +2071,7 @@
         <v>66</v>
       </c>
       <c r="E85">
-        <v>100</v>
+        <v>38.38383838383839</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -2088,7 +2088,7 @@
         <v>65</v>
       </c>
       <c r="E86">
-        <v>68.9655172413793</v>
+        <v>31.48148148148148</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -2105,7 +2105,7 @@
         <v>66</v>
       </c>
       <c r="E87">
-        <v>74.07407407407408</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -2122,7 +2122,7 @@
         <v>67</v>
       </c>
       <c r="E88">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -2139,7 +2139,7 @@
         <v>68</v>
       </c>
       <c r="E89">
-        <v>71.42857142857143</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -2156,7 +2156,7 @@
         <v>69</v>
       </c>
       <c r="E90">
-        <v>70.17543859649123</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -2173,7 +2173,7 @@
         <v>70</v>
       </c>
       <c r="E91">
-        <v>35.18518518518519</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -2190,7 +2190,7 @@
         <v>71</v>
       </c>
       <c r="E92">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -2207,7 +2207,7 @@
         <v>72</v>
       </c>
       <c r="E93">
-        <v>33.64485981308411</v>
+        <v>28.0373831775701</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -2224,7 +2224,7 @@
         <v>73</v>
       </c>
       <c r="E94">
-        <v>31.68316831683168</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -2241,7 +2241,7 @@
         <v>74</v>
       </c>
       <c r="E95">
-        <v>35.64356435643565</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -2258,7 +2258,7 @@
         <v>75</v>
       </c>
       <c r="E96">
-        <v>33.33333333333333</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2275,7 +2275,7 @@
         <v>76</v>
       </c>
       <c r="E97">
-        <v>33.00970873786407</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -2292,7 +2292,7 @@
         <v>77</v>
       </c>
       <c r="E98">
-        <v>30.3030303030303</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2309,7 +2309,7 @@
         <v>78</v>
       </c>
       <c r="E99">
-        <v>34.95145631067962</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -2326,7 +2326,7 @@
         <v>79</v>
       </c>
       <c r="E100">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -2343,7 +2343,7 @@
         <v>80</v>
       </c>
       <c r="E101">
-        <v>30.76923076923077</v>
+        <v>26.92307692307693</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2360,7 +2360,7 @@
         <v>81</v>
       </c>
       <c r="E102">
-        <v>27.72277227722772</v>
+        <v>23.76237623762376</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -2377,7 +2377,7 @@
         <v>82</v>
       </c>
       <c r="E103">
-        <v>31.77570093457943</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2394,7 +2394,7 @@
         <v>83</v>
       </c>
       <c r="E104">
-        <v>30.18867924528301</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -2411,7 +2411,7 @@
         <v>84</v>
       </c>
       <c r="E105">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -2428,7 +2428,7 @@
         <v>67</v>
       </c>
       <c r="E106">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -2445,7 +2445,7 @@
         <v>65</v>
       </c>
       <c r="E107">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -2462,7 +2462,7 @@
         <v>66</v>
       </c>
       <c r="E108">
-        <v>74.07407407407408</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2479,7 +2479,7 @@
         <v>67</v>
       </c>
       <c r="E109">
-        <v>68.9655172413793</v>
+        <v>31.48148148148148</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -2496,7 +2496,7 @@
         <v>68</v>
       </c>
       <c r="E110">
-        <v>71.42857142857143</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -2513,7 +2513,7 @@
         <v>69</v>
       </c>
       <c r="E111">
-        <v>70.17543859649123</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2530,7 +2530,7 @@
         <v>70</v>
       </c>
       <c r="E112">
-        <v>31.48148148148148</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -2547,7 +2547,7 @@
         <v>71</v>
       </c>
       <c r="E113">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -2564,7 +2564,7 @@
         <v>72</v>
       </c>
       <c r="E114">
-        <v>33.64485981308411</v>
+        <v>28.0373831775701</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -2581,7 +2581,7 @@
         <v>73</v>
       </c>
       <c r="E115">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -2598,7 +2598,7 @@
         <v>74</v>
       </c>
       <c r="E116">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -2615,7 +2615,7 @@
         <v>75</v>
       </c>
       <c r="E117">
-        <v>29.41176470588235</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -2632,7 +2632,7 @@
         <v>76</v>
       </c>
       <c r="E118">
-        <v>31.06796116504854</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -2649,7 +2649,7 @@
         <v>77</v>
       </c>
       <c r="E119">
-        <v>28.28282828282828</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -2666,7 +2666,7 @@
         <v>78</v>
       </c>
       <c r="E120">
-        <v>33.00970873786407</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -2683,7 +2683,7 @@
         <v>79</v>
       </c>
       <c r="E121">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -2700,7 +2700,7 @@
         <v>80</v>
       </c>
       <c r="E122">
-        <v>74.07407407407408</v>
+        <v>42.30769230769231</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -2717,7 +2717,7 @@
         <v>81</v>
       </c>
       <c r="E123">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -2734,7 +2734,7 @@
         <v>82</v>
       </c>
       <c r="E124">
-        <v>31.77570093457943</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -2751,7 +2751,7 @@
         <v>83</v>
       </c>
       <c r="E125">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -2768,7 +2768,7 @@
         <v>84</v>
       </c>
       <c r="E126">
-        <v>31.68316831683168</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -2785,7 +2785,7 @@
         <v>65</v>
       </c>
       <c r="E127">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -2802,7 +2802,7 @@
         <v>65</v>
       </c>
       <c r="E128">
-        <v>68.9655172413793</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -2819,7 +2819,7 @@
         <v>66</v>
       </c>
       <c r="E129">
-        <v>74.07407407407408</v>
+        <v>33.66336633663366</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -2836,7 +2836,7 @@
         <v>67</v>
       </c>
       <c r="E130">
-        <v>68.9655172413793</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -2853,7 +2853,7 @@
         <v>68</v>
       </c>
       <c r="E131">
-        <v>100</v>
+        <v>40.77669902912622</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -2870,7 +2870,7 @@
         <v>69</v>
       </c>
       <c r="E132">
-        <v>70.17543859649123</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -2887,7 +2887,7 @@
         <v>70</v>
       </c>
       <c r="E133">
-        <v>34.28571428571429</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -2904,7 +2904,7 @@
         <v>71</v>
       </c>
       <c r="E134">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -2921,7 +2921,7 @@
         <v>72</v>
       </c>
       <c r="E135">
-        <v>36.53846153846154</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2938,7 +2938,7 @@
         <v>73</v>
       </c>
       <c r="E136">
-        <v>34.69387755102041</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -2955,7 +2955,7 @@
         <v>74</v>
       </c>
       <c r="E137">
-        <v>32.65306122448979</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -2972,7 +2972,7 @@
         <v>75</v>
       </c>
       <c r="E138">
-        <v>34.34343434343434</v>
+        <v>30.3030303030303</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -2989,7 +2989,7 @@
         <v>76</v>
       </c>
       <c r="E139">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -3006,7 +3006,7 @@
         <v>77</v>
       </c>
       <c r="E140">
-        <v>31.25</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -3023,7 +3023,7 @@
         <v>78</v>
       </c>
       <c r="E141">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -3040,7 +3040,7 @@
         <v>79</v>
       </c>
       <c r="E142">
-        <v>33.00970873786407</v>
+        <v>29.12621359223301</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -3057,7 +3057,7 @@
         <v>80</v>
       </c>
       <c r="E143">
-        <v>33.66336633663366</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -3074,7 +3074,7 @@
         <v>81</v>
       </c>
       <c r="E144">
-        <v>32.65306122448979</v>
+        <v>26.53061224489796</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -3091,7 +3091,7 @@
         <v>82</v>
       </c>
       <c r="E145">
-        <v>36.53846153846154</v>
+        <v>28.84615384615384</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -3108,7 +3108,7 @@
         <v>83</v>
       </c>
       <c r="E146">
-        <v>38.83495145631068</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -3125,7 +3125,7 @@
         <v>84</v>
       </c>
       <c r="E147">
-        <v>34.69387755102041</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -3142,7 +3142,7 @@
         <v>68</v>
       </c>
       <c r="E148">
-        <v>100</v>
+        <v>40.77669902912622</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -3159,7 +3159,7 @@
         <v>65</v>
       </c>
       <c r="E149">
-        <v>68.9655172413793</v>
+        <v>31.48148148148148</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -3176,7 +3176,7 @@
         <v>66</v>
       </c>
       <c r="E150">
-        <v>74.07407407407408</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -3193,7 +3193,7 @@
         <v>67</v>
       </c>
       <c r="E151">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -3210,7 +3210,7 @@
         <v>68</v>
       </c>
       <c r="E152">
-        <v>71.42857142857143</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -3227,7 +3227,7 @@
         <v>69</v>
       </c>
       <c r="E153">
-        <v>70.17543859649123</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -3244,7 +3244,7 @@
         <v>70</v>
       </c>
       <c r="E154">
-        <v>35.18518518518519</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -3261,7 +3261,7 @@
         <v>71</v>
       </c>
       <c r="E155">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -3278,7 +3278,7 @@
         <v>72</v>
       </c>
       <c r="E156">
-        <v>33.64485981308411</v>
+        <v>28.0373831775701</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -3295,7 +3295,7 @@
         <v>73</v>
       </c>
       <c r="E157">
-        <v>31.68316831683168</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -3312,7 +3312,7 @@
         <v>74</v>
       </c>
       <c r="E158">
-        <v>35.64356435643565</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -3329,7 +3329,7 @@
         <v>75</v>
       </c>
       <c r="E159">
-        <v>33.33333333333333</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -3346,7 +3346,7 @@
         <v>76</v>
       </c>
       <c r="E160">
-        <v>33.00970873786407</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -3363,7 +3363,7 @@
         <v>77</v>
       </c>
       <c r="E161">
-        <v>30.3030303030303</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -3380,7 +3380,7 @@
         <v>78</v>
       </c>
       <c r="E162">
-        <v>34.95145631067962</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -3397,7 +3397,7 @@
         <v>79</v>
       </c>
       <c r="E163">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -3414,7 +3414,7 @@
         <v>80</v>
       </c>
       <c r="E164">
-        <v>30.76923076923077</v>
+        <v>26.92307692307693</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -3431,7 +3431,7 @@
         <v>81</v>
       </c>
       <c r="E165">
-        <v>27.72277227722772</v>
+        <v>23.76237623762376</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -3448,7 +3448,7 @@
         <v>82</v>
       </c>
       <c r="E166">
-        <v>31.77570093457943</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -3465,7 +3465,7 @@
         <v>83</v>
       </c>
       <c r="E167">
-        <v>30.18867924528301</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -3482,7 +3482,7 @@
         <v>84</v>
       </c>
       <c r="E168">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -3499,7 +3499,7 @@
         <v>67</v>
       </c>
       <c r="E169">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -3516,7 +3516,7 @@
         <v>65</v>
       </c>
       <c r="E170">
-        <v>68.9655172413793</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -3533,7 +3533,7 @@
         <v>66</v>
       </c>
       <c r="E171">
-        <v>74.07407407407408</v>
+        <v>33.66336633663366</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -3550,7 +3550,7 @@
         <v>67</v>
       </c>
       <c r="E172">
-        <v>68.9655172413793</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -3567,7 +3567,7 @@
         <v>68</v>
       </c>
       <c r="E173">
-        <v>100</v>
+        <v>40.77669902912622</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -3584,7 +3584,7 @@
         <v>69</v>
       </c>
       <c r="E174">
-        <v>70.17543859649123</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -3601,7 +3601,7 @@
         <v>70</v>
       </c>
       <c r="E175">
-        <v>34.28571428571429</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -3618,7 +3618,7 @@
         <v>71</v>
       </c>
       <c r="E176">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="177" spans="1:5">
@@ -3635,7 +3635,7 @@
         <v>72</v>
       </c>
       <c r="E177">
-        <v>36.53846153846154</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -3652,7 +3652,7 @@
         <v>73</v>
       </c>
       <c r="E178">
-        <v>34.69387755102041</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -3669,7 +3669,7 @@
         <v>74</v>
       </c>
       <c r="E179">
-        <v>32.65306122448979</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -3686,7 +3686,7 @@
         <v>75</v>
       </c>
       <c r="E180">
-        <v>34.34343434343434</v>
+        <v>30.3030303030303</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -3703,7 +3703,7 @@
         <v>76</v>
       </c>
       <c r="E181">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="182" spans="1:5">
@@ -3720,7 +3720,7 @@
         <v>77</v>
       </c>
       <c r="E182">
-        <v>31.25</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -3737,7 +3737,7 @@
         <v>78</v>
       </c>
       <c r="E183">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="184" spans="1:5">
@@ -3754,7 +3754,7 @@
         <v>79</v>
       </c>
       <c r="E184">
-        <v>33.00970873786407</v>
+        <v>29.12621359223301</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -3771,7 +3771,7 @@
         <v>80</v>
       </c>
       <c r="E185">
-        <v>33.66336633663366</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -3788,7 +3788,7 @@
         <v>81</v>
       </c>
       <c r="E186">
-        <v>32.65306122448979</v>
+        <v>26.53061224489796</v>
       </c>
     </row>
     <row r="187" spans="1:5">
@@ -3805,7 +3805,7 @@
         <v>82</v>
       </c>
       <c r="E187">
-        <v>36.53846153846154</v>
+        <v>28.84615384615384</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -3822,7 +3822,7 @@
         <v>83</v>
       </c>
       <c r="E188">
-        <v>38.83495145631068</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -3839,7 +3839,7 @@
         <v>84</v>
       </c>
       <c r="E189">
-        <v>34.69387755102041</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -3856,7 +3856,7 @@
         <v>68</v>
       </c>
       <c r="E190">
-        <v>100</v>
+        <v>40.77669902912622</v>
       </c>
     </row>
     <row r="191" spans="1:5">
@@ -3873,7 +3873,7 @@
         <v>65</v>
       </c>
       <c r="E191">
-        <v>68.9655172413793</v>
+        <v>31.48148148148148</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -3890,7 +3890,7 @@
         <v>66</v>
       </c>
       <c r="E192">
-        <v>74.07407407407408</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -3907,7 +3907,7 @@
         <v>67</v>
       </c>
       <c r="E193">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -3924,7 +3924,7 @@
         <v>68</v>
       </c>
       <c r="E194">
-        <v>71.42857142857143</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -3941,7 +3941,7 @@
         <v>69</v>
       </c>
       <c r="E195">
-        <v>70.17543859649123</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -3958,7 +3958,7 @@
         <v>70</v>
       </c>
       <c r="E196">
-        <v>35.18518518518519</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -3975,7 +3975,7 @@
         <v>71</v>
       </c>
       <c r="E197">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -3992,7 +3992,7 @@
         <v>72</v>
       </c>
       <c r="E198">
-        <v>33.64485981308411</v>
+        <v>28.0373831775701</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -4009,7 +4009,7 @@
         <v>73</v>
       </c>
       <c r="E199">
-        <v>31.68316831683168</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -4026,7 +4026,7 @@
         <v>74</v>
       </c>
       <c r="E200">
-        <v>35.64356435643565</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -4043,7 +4043,7 @@
         <v>75</v>
       </c>
       <c r="E201">
-        <v>33.33333333333333</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -4060,7 +4060,7 @@
         <v>76</v>
       </c>
       <c r="E202">
-        <v>33.00970873786407</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -4077,7 +4077,7 @@
         <v>77</v>
       </c>
       <c r="E203">
-        <v>30.3030303030303</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -4094,7 +4094,7 @@
         <v>78</v>
       </c>
       <c r="E204">
-        <v>34.95145631067962</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -4111,7 +4111,7 @@
         <v>79</v>
       </c>
       <c r="E205">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -4128,7 +4128,7 @@
         <v>80</v>
       </c>
       <c r="E206">
-        <v>30.76923076923077</v>
+        <v>26.92307692307693</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -4145,7 +4145,7 @@
         <v>81</v>
       </c>
       <c r="E207">
-        <v>27.72277227722772</v>
+        <v>23.76237623762376</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -4162,7 +4162,7 @@
         <v>82</v>
       </c>
       <c r="E208">
-        <v>31.77570093457943</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -4179,7 +4179,7 @@
         <v>83</v>
       </c>
       <c r="E209">
-        <v>30.18867924528301</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -4196,7 +4196,7 @@
         <v>84</v>
       </c>
       <c r="E210">
-        <v>29.70297029702971</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -4213,7 +4213,7 @@
         <v>67</v>
       </c>
       <c r="E211">
-        <v>100</v>
+        <v>42.5925925925926</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -4230,7 +4230,7 @@
         <v>65</v>
       </c>
       <c r="E212">
-        <v>68.9655172413793</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -4247,7 +4247,7 @@
         <v>66</v>
       </c>
       <c r="E213">
-        <v>74.07407407407408</v>
+        <v>33.33333333333334</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -4264,7 +4264,7 @@
         <v>67</v>
       </c>
       <c r="E214">
-        <v>68.9655172413793</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -4281,7 +4281,7 @@
         <v>68</v>
       </c>
       <c r="E215">
-        <v>71.42857142857143</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -4298,7 +4298,7 @@
         <v>69</v>
       </c>
       <c r="E216">
-        <v>100</v>
+        <v>41.9047619047619</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -4315,7 +4315,7 @@
         <v>70</v>
       </c>
       <c r="E217">
-        <v>28.30188679245283</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -4332,7 +4332,7 @@
         <v>71</v>
       </c>
       <c r="E218">
-        <v>53.65853658536585</v>
+        <v>32.6530612244898</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -4349,7 +4349,7 @@
         <v>72</v>
       </c>
       <c r="E219">
-        <v>32.38095238095238</v>
+        <v>26.66666666666667</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -4366,7 +4366,7 @@
         <v>73</v>
       </c>
       <c r="E220">
-        <v>32.32323232323232</v>
+        <v>24.24242424242424</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -4383,7 +4383,7 @@
         <v>74</v>
       </c>
       <c r="E221">
-        <v>28.28282828282828</v>
+        <v>24.24242424242424</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -4400,7 +4400,7 @@
         <v>75</v>
       </c>
       <c r="E222">
-        <v>30</v>
+        <v>24</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -4417,7 +4417,7 @@
         <v>76</v>
       </c>
       <c r="E223">
-        <v>31.68316831683168</v>
+        <v>27.72277227722773</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -4434,7 +4434,7 @@
         <v>77</v>
       </c>
       <c r="E224">
-        <v>28.8659793814433</v>
+        <v>20.61855670103093</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -4451,7 +4451,7 @@
         <v>78</v>
       </c>
       <c r="E225">
-        <v>33.66336633663366</v>
+        <v>27.72277227722773</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -4468,7 +4468,7 @@
         <v>79</v>
       </c>
       <c r="E226">
-        <v>30.76923076923077</v>
+        <v>26.92307692307693</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -4485,7 +4485,7 @@
         <v>80</v>
       </c>
       <c r="E227">
-        <v>33.33333333333333</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -4502,7 +4502,7 @@
         <v>81</v>
       </c>
       <c r="E228">
-        <v>30.3030303030303</v>
+        <v>22.22222222222222</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -4519,7 +4519,7 @@
         <v>82</v>
       </c>
       <c r="E229">
-        <v>32.38095238095238</v>
+        <v>24.76190476190476</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -4536,7 +4536,7 @@
         <v>83</v>
       </c>
       <c r="E230">
-        <v>34.61538461538461</v>
+        <v>25</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -4553,7 +4553,7 @@
         <v>84</v>
       </c>
       <c r="E231">
-        <v>32.32323232323232</v>
+        <v>26.26262626262627</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -4570,7 +4570,7 @@
         <v>69</v>
       </c>
       <c r="E232">
-        <v>100</v>
+        <v>41.9047619047619</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -4587,7 +4587,7 @@
         <v>65</v>
       </c>
       <c r="E233">
-        <v>68.9655172413793</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -4604,7 +4604,7 @@
         <v>66</v>
       </c>
       <c r="E234">
-        <v>74.07407407407408</v>
+        <v>33.66336633663366</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -4621,7 +4621,7 @@
         <v>67</v>
       </c>
       <c r="E235">
-        <v>68.9655172413793</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -4638,7 +4638,7 @@
         <v>68</v>
       </c>
       <c r="E236">
-        <v>100</v>
+        <v>40.77669902912622</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -4655,7 +4655,7 @@
         <v>69</v>
       </c>
       <c r="E237">
-        <v>70.17543859649123</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -4672,7 +4672,7 @@
         <v>70</v>
       </c>
       <c r="E238">
-        <v>34.28571428571429</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="239" spans="1:5">
@@ -4689,7 +4689,7 @@
         <v>71</v>
       </c>
       <c r="E239">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="240" spans="1:5">
@@ -4706,7 +4706,7 @@
         <v>72</v>
       </c>
       <c r="E240">
-        <v>36.53846153846154</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -4723,7 +4723,7 @@
         <v>73</v>
       </c>
       <c r="E241">
-        <v>34.69387755102041</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -4740,7 +4740,7 @@
         <v>74</v>
       </c>
       <c r="E242">
-        <v>32.65306122448979</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="243" spans="1:5">
@@ -4757,7 +4757,7 @@
         <v>75</v>
       </c>
       <c r="E243">
-        <v>34.34343434343434</v>
+        <v>30.3030303030303</v>
       </c>
     </row>
     <row r="244" spans="1:5">
@@ -4774,7 +4774,7 @@
         <v>76</v>
       </c>
       <c r="E244">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="245" spans="1:5">
@@ -4791,7 +4791,7 @@
         <v>77</v>
       </c>
       <c r="E245">
-        <v>31.25</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="246" spans="1:5">
@@ -4808,7 +4808,7 @@
         <v>78</v>
       </c>
       <c r="E246">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="247" spans="1:5">
@@ -4825,7 +4825,7 @@
         <v>79</v>
       </c>
       <c r="E247">
-        <v>33.00970873786407</v>
+        <v>29.12621359223301</v>
       </c>
     </row>
     <row r="248" spans="1:5">
@@ -4842,7 +4842,7 @@
         <v>80</v>
       </c>
       <c r="E248">
-        <v>33.66336633663366</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="249" spans="1:5">
@@ -4859,7 +4859,7 @@
         <v>81</v>
       </c>
       <c r="E249">
-        <v>32.65306122448979</v>
+        <v>26.53061224489796</v>
       </c>
     </row>
     <row r="250" spans="1:5">
@@ -4876,7 +4876,7 @@
         <v>82</v>
       </c>
       <c r="E250">
-        <v>36.53846153846154</v>
+        <v>28.84615384615384</v>
       </c>
     </row>
     <row r="251" spans="1:5">
@@ -4893,7 +4893,7 @@
         <v>83</v>
       </c>
       <c r="E251">
-        <v>38.83495145631068</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="252" spans="1:5">
@@ -4910,7 +4910,7 @@
         <v>84</v>
       </c>
       <c r="E252">
-        <v>34.69387755102041</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="253" spans="1:5">
@@ -4927,7 +4927,7 @@
         <v>68</v>
       </c>
       <c r="E253">
-        <v>100</v>
+        <v>40.77669902912622</v>
       </c>
     </row>
     <row r="254" spans="1:5">
@@ -4944,7 +4944,7 @@
         <v>65</v>
       </c>
       <c r="E254">
-        <v>68.9655172413793</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="255" spans="1:5">
@@ -4961,7 +4961,7 @@
         <v>66</v>
       </c>
       <c r="E255">
-        <v>74.07407407407408</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="256" spans="1:5">
@@ -4978,7 +4978,7 @@
         <v>67</v>
       </c>
       <c r="E256">
-        <v>68.9655172413793</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="257" spans="1:5">
@@ -4995,7 +4995,7 @@
         <v>68</v>
       </c>
       <c r="E257">
-        <v>71.42857142857143</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="258" spans="1:5">
@@ -5012,7 +5012,7 @@
         <v>69</v>
       </c>
       <c r="E258">
-        <v>100</v>
+        <v>41.50943396226415</v>
       </c>
     </row>
     <row r="259" spans="1:5">
@@ -5029,7 +5029,7 @@
         <v>70</v>
       </c>
       <c r="E259">
-        <v>28.03738317757009</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="260" spans="1:5">
@@ -5046,7 +5046,7 @@
         <v>71</v>
       </c>
       <c r="E260">
-        <v>53.65853658536585</v>
+        <v>32.32323232323232</v>
       </c>
     </row>
     <row r="261" spans="1:5">
@@ -5063,7 +5063,7 @@
         <v>72</v>
       </c>
       <c r="E261">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="262" spans="1:5">
@@ -5080,7 +5080,7 @@
         <v>73</v>
       </c>
       <c r="E262">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="263" spans="1:5">
@@ -5097,7 +5097,7 @@
         <v>74</v>
       </c>
       <c r="E263">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="264" spans="1:5">
@@ -5114,7 +5114,7 @@
         <v>75</v>
       </c>
       <c r="E264">
-        <v>29.70297029702971</v>
+        <v>23.76237623762376</v>
       </c>
     </row>
     <row r="265" spans="1:5">
@@ -5131,7 +5131,7 @@
         <v>76</v>
       </c>
       <c r="E265">
-        <v>31.37254901960785</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="266" spans="1:5">
@@ -5148,7 +5148,7 @@
         <v>77</v>
       </c>
       <c r="E266">
-        <v>28.57142857142857</v>
+        <v>20.40816326530612</v>
       </c>
     </row>
     <row r="267" spans="1:5">
@@ -5165,7 +5165,7 @@
         <v>78</v>
       </c>
       <c r="E267">
-        <v>33.33333333333333</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="268" spans="1:5">
@@ -5182,7 +5182,7 @@
         <v>79</v>
       </c>
       <c r="E268">
-        <v>30.47619047619048</v>
+        <v>26.66666666666667</v>
       </c>
     </row>
     <row r="269" spans="1:5">
@@ -5199,7 +5199,7 @@
         <v>80</v>
       </c>
       <c r="E269">
-        <v>33.00970873786407</v>
+        <v>25.24271844660194</v>
       </c>
     </row>
     <row r="270" spans="1:5">
@@ -5216,7 +5216,7 @@
         <v>81</v>
       </c>
       <c r="E270">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="271" spans="1:5">
@@ -5233,7 +5233,7 @@
         <v>82</v>
       </c>
       <c r="E271">
-        <v>32.0754716981132</v>
+        <v>24.52830188679245</v>
       </c>
     </row>
     <row r="272" spans="1:5">
@@ -5250,7 +5250,7 @@
         <v>83</v>
       </c>
       <c r="E272">
-        <v>34.28571428571429</v>
+        <v>24.76190476190476</v>
       </c>
     </row>
     <row r="273" spans="1:5">
@@ -5267,7 +5267,7 @@
         <v>84</v>
       </c>
       <c r="E273">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="274" spans="1:5">
@@ -5284,7 +5284,7 @@
         <v>69</v>
       </c>
       <c r="E274">
-        <v>100</v>
+        <v>41.50943396226415</v>
       </c>
     </row>
     <row r="275" spans="1:5">
@@ -5301,7 +5301,7 @@
         <v>65</v>
       </c>
       <c r="E275">
-        <v>68.9655172413793</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="276" spans="1:5">
@@ -5318,7 +5318,7 @@
         <v>66</v>
       </c>
       <c r="E276">
-        <v>74.07407407407408</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="277" spans="1:5">
@@ -5335,7 +5335,7 @@
         <v>67</v>
       </c>
       <c r="E277">
-        <v>68.9655172413793</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="278" spans="1:5">
@@ -5352,7 +5352,7 @@
         <v>68</v>
       </c>
       <c r="E278">
-        <v>71.42857142857143</v>
+        <v>32.38095238095238</v>
       </c>
     </row>
     <row r="279" spans="1:5">
@@ -5369,7 +5369,7 @@
         <v>69</v>
       </c>
       <c r="E279">
-        <v>100</v>
+        <v>41.50943396226415</v>
       </c>
     </row>
     <row r="280" spans="1:5">
@@ -5386,7 +5386,7 @@
         <v>70</v>
       </c>
       <c r="E280">
-        <v>28.03738317757009</v>
+        <v>26.16822429906542</v>
       </c>
     </row>
     <row r="281" spans="1:5">
@@ -5403,7 +5403,7 @@
         <v>71</v>
       </c>
       <c r="E281">
-        <v>53.65853658536585</v>
+        <v>32.32323232323232</v>
       </c>
     </row>
     <row r="282" spans="1:5">
@@ -5420,7 +5420,7 @@
         <v>72</v>
       </c>
       <c r="E282">
-        <v>32.0754716981132</v>
+        <v>26.41509433962265</v>
       </c>
     </row>
     <row r="283" spans="1:5">
@@ -5437,7 +5437,7 @@
         <v>73</v>
       </c>
       <c r="E283">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="284" spans="1:5">
@@ -5454,7 +5454,7 @@
         <v>74</v>
       </c>
       <c r="E284">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="285" spans="1:5">
@@ -5471,7 +5471,7 @@
         <v>75</v>
       </c>
       <c r="E285">
-        <v>29.70297029702971</v>
+        <v>23.76237623762376</v>
       </c>
     </row>
     <row r="286" spans="1:5">
@@ -5488,7 +5488,7 @@
         <v>76</v>
       </c>
       <c r="E286">
-        <v>31.37254901960785</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="287" spans="1:5">
@@ -5505,7 +5505,7 @@
         <v>77</v>
       </c>
       <c r="E287">
-        <v>28.57142857142857</v>
+        <v>20.40816326530612</v>
       </c>
     </row>
     <row r="288" spans="1:5">
@@ -5522,7 +5522,7 @@
         <v>78</v>
       </c>
       <c r="E288">
-        <v>33.33333333333333</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="289" spans="1:5">
@@ -5539,7 +5539,7 @@
         <v>79</v>
       </c>
       <c r="E289">
-        <v>30.47619047619048</v>
+        <v>26.66666666666667</v>
       </c>
     </row>
     <row r="290" spans="1:5">
@@ -5556,7 +5556,7 @@
         <v>80</v>
       </c>
       <c r="E290">
-        <v>33.00970873786407</v>
+        <v>25.24271844660194</v>
       </c>
     </row>
     <row r="291" spans="1:5">
@@ -5573,7 +5573,7 @@
         <v>81</v>
       </c>
       <c r="E291">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="292" spans="1:5">
@@ -5590,7 +5590,7 @@
         <v>82</v>
       </c>
       <c r="E292">
-        <v>32.0754716981132</v>
+        <v>24.52830188679245</v>
       </c>
     </row>
     <row r="293" spans="1:5">
@@ -5607,7 +5607,7 @@
         <v>83</v>
       </c>
       <c r="E293">
-        <v>34.28571428571429</v>
+        <v>24.76190476190476</v>
       </c>
     </row>
     <row r="294" spans="1:5">
@@ -5624,7 +5624,7 @@
         <v>84</v>
       </c>
       <c r="E294">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="295" spans="1:5">
@@ -5641,7 +5641,7 @@
         <v>69</v>
       </c>
       <c r="E295">
-        <v>100</v>
+        <v>41.50943396226415</v>
       </c>
     </row>
     <row r="296" spans="1:5">
@@ -5658,7 +5658,7 @@
         <v>65</v>
       </c>
       <c r="E296">
-        <v>68.9655172413793</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="297" spans="1:5">
@@ -5675,7 +5675,7 @@
         <v>66</v>
       </c>
       <c r="E297">
-        <v>100</v>
+        <v>38.38383838383839</v>
       </c>
     </row>
     <row r="298" spans="1:5">
@@ -5692,7 +5692,7 @@
         <v>67</v>
       </c>
       <c r="E298">
-        <v>68.9655172413793</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="299" spans="1:5">
@@ -5709,7 +5709,7 @@
         <v>68</v>
       </c>
       <c r="E299">
-        <v>71.42857142857143</v>
+        <v>33.66336633663366</v>
       </c>
     </row>
     <row r="300" spans="1:5">
@@ -5726,7 +5726,7 @@
         <v>69</v>
       </c>
       <c r="E300">
-        <v>70.17543859649123</v>
+        <v>33.33333333333334</v>
       </c>
     </row>
     <row r="301" spans="1:5">
@@ -5743,7 +5743,7 @@
         <v>70</v>
       </c>
       <c r="E301">
-        <v>33.00970873786407</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="302" spans="1:5">
@@ -5760,7 +5760,7 @@
         <v>71</v>
       </c>
       <c r="E302">
-        <v>31.57894736842105</v>
+        <v>27.36842105263158</v>
       </c>
     </row>
     <row r="303" spans="1:5">
@@ -5777,7 +5777,7 @@
         <v>72</v>
       </c>
       <c r="E303">
-        <v>33.33333333333333</v>
+        <v>31.37254901960784</v>
       </c>
     </row>
     <row r="304" spans="1:5">
@@ -5794,7 +5794,7 @@
         <v>73</v>
       </c>
       <c r="E304">
-        <v>31.25</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="305" spans="1:5">
@@ -5811,7 +5811,7 @@
         <v>74</v>
       </c>
       <c r="E305">
-        <v>33.33333333333333</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="306" spans="1:5">
@@ -5828,7 +5828,7 @@
         <v>75</v>
       </c>
       <c r="E306">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="307" spans="1:5">
@@ -5845,7 +5845,7 @@
         <v>76</v>
       </c>
       <c r="E307">
-        <v>32.65306122448979</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="308" spans="1:5">
@@ -5862,7 +5862,7 @@
         <v>77</v>
       </c>
       <c r="E308">
-        <v>29.78723404255319</v>
+        <v>25.53191489361702</v>
       </c>
     </row>
     <row r="309" spans="1:5">
@@ -5879,7 +5879,7 @@
         <v>78</v>
       </c>
       <c r="E309">
-        <v>36.73469387755102</v>
+        <v>30.61224489795918</v>
       </c>
     </row>
     <row r="310" spans="1:5">
@@ -5896,7 +5896,7 @@
         <v>79</v>
       </c>
       <c r="E310">
-        <v>35.64356435643565</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="311" spans="1:5">
@@ -5913,7 +5913,7 @@
         <v>80</v>
       </c>
       <c r="E311">
-        <v>34.34343434343434</v>
+        <v>28.28282828282829</v>
       </c>
     </row>
     <row r="312" spans="1:5">
@@ -5930,7 +5930,7 @@
         <v>81</v>
       </c>
       <c r="E312">
-        <v>33.33333333333333</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="313" spans="1:5">
@@ -5947,7 +5947,7 @@
         <v>82</v>
       </c>
       <c r="E313">
-        <v>31.37254901960785</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="314" spans="1:5">
@@ -5964,7 +5964,7 @@
         <v>83</v>
       </c>
       <c r="E314">
-        <v>31.68316831683168</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="315" spans="1:5">
@@ -5981,7 +5981,7 @@
         <v>84</v>
       </c>
       <c r="E315">
-        <v>33.33333333333333</v>
+        <v>29.16666666666666</v>
       </c>
     </row>
     <row r="316" spans="1:5">
@@ -5998,7 +5998,7 @@
         <v>66</v>
       </c>
       <c r="E316">
-        <v>100</v>
+        <v>38.38383838383839</v>
       </c>
     </row>
     <row r="317" spans="1:5">
@@ -6015,7 +6015,7 @@
         <v>65</v>
       </c>
       <c r="E317">
-        <v>68.9655172413793</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="318" spans="1:5">
@@ -6032,7 +6032,7 @@
         <v>66</v>
       </c>
       <c r="E318">
-        <v>100</v>
+        <v>38</v>
       </c>
     </row>
     <row r="319" spans="1:5">
@@ -6049,7 +6049,7 @@
         <v>67</v>
       </c>
       <c r="E319">
-        <v>68.9655172413793</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="320" spans="1:5">
@@ -6066,7 +6066,7 @@
         <v>68</v>
       </c>
       <c r="E320">
-        <v>71.42857142857143</v>
+        <v>33.33333333333334</v>
       </c>
     </row>
     <row r="321" spans="1:5">
@@ -6083,7 +6083,7 @@
         <v>69</v>
       </c>
       <c r="E321">
-        <v>70.17543859649123</v>
+        <v>33.00970873786407</v>
       </c>
     </row>
     <row r="322" spans="1:5">
@@ -6100,7 +6100,7 @@
         <v>70</v>
       </c>
       <c r="E322">
-        <v>32.69230769230769</v>
+        <v>30.76923076923077</v>
       </c>
     </row>
     <row r="323" spans="1:5">
@@ -6117,7 +6117,7 @@
         <v>71</v>
       </c>
       <c r="E323">
-        <v>31.25</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="324" spans="1:5">
@@ -6134,7 +6134,7 @@
         <v>72</v>
       </c>
       <c r="E324">
-        <v>33.00970873786407</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="325" spans="1:5">
@@ -6151,7 +6151,7 @@
         <v>73</v>
       </c>
       <c r="E325">
-        <v>30.9278350515464</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="326" spans="1:5">
@@ -6168,7 +6168,7 @@
         <v>74</v>
       </c>
       <c r="E326">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="327" spans="1:5">
@@ -6185,7 +6185,7 @@
         <v>75</v>
       </c>
       <c r="E327">
-        <v>32.65306122448979</v>
+        <v>28.57142857142857</v>
       </c>
     </row>
     <row r="328" spans="1:5">
@@ -6202,7 +6202,7 @@
         <v>76</v>
       </c>
       <c r="E328">
-        <v>32.32323232323232</v>
+        <v>30.3030303030303</v>
       </c>
     </row>
     <row r="329" spans="1:5">
@@ -6219,7 +6219,7 @@
         <v>77</v>
       </c>
       <c r="E329">
-        <v>29.47368421052632</v>
+        <v>25.26315789473684</v>
       </c>
     </row>
     <row r="330" spans="1:5">
@@ -6236,7 +6236,7 @@
         <v>78</v>
       </c>
       <c r="E330">
-        <v>36.36363636363637</v>
+        <v>30.3030303030303</v>
       </c>
     </row>
     <row r="331" spans="1:5">
@@ -6253,7 +6253,7 @@
         <v>79</v>
       </c>
       <c r="E331">
-        <v>35.29411764705883</v>
+        <v>29.41176470588235</v>
       </c>
     </row>
     <row r="332" spans="1:5">
@@ -6270,7 +6270,7 @@
         <v>80</v>
       </c>
       <c r="E332">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="333" spans="1:5">
@@ -6287,7 +6287,7 @@
         <v>81</v>
       </c>
       <c r="E333">
-        <v>32.98969072164948</v>
+        <v>26.80412371134021</v>
       </c>
     </row>
     <row r="334" spans="1:5">
@@ -6304,7 +6304,7 @@
         <v>82</v>
       </c>
       <c r="E334">
-        <v>31.06796116504854</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="335" spans="1:5">
@@ -6321,7 +6321,7 @@
         <v>83</v>
       </c>
       <c r="E335">
-        <v>31.37254901960785</v>
+        <v>29.41176470588235</v>
       </c>
     </row>
     <row r="336" spans="1:5">
@@ -6338,7 +6338,7 @@
         <v>84</v>
       </c>
       <c r="E336">
-        <v>32.98969072164948</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="337" spans="1:5">
@@ -6355,7 +6355,7 @@
         <v>66</v>
       </c>
       <c r="E337">
-        <v>100</v>
+        <v>38</v>
       </c>
     </row>
     <row r="338" spans="1:5">
@@ -6372,7 +6372,7 @@
         <v>65</v>
       </c>
       <c r="E338">
-        <v>34.86238532110092</v>
+        <v>25.68807339449542</v>
       </c>
     </row>
     <row r="339" spans="1:5">
@@ -6389,7 +6389,7 @@
         <v>66</v>
       </c>
       <c r="E339">
-        <v>34.28571428571429</v>
+        <v>28.57142857142857</v>
       </c>
     </row>
     <row r="340" spans="1:5">
@@ -6406,7 +6406,7 @@
         <v>67</v>
       </c>
       <c r="E340">
-        <v>33.02752293577981</v>
+        <v>31.19266055045872</v>
       </c>
     </row>
     <row r="341" spans="1:5">
@@ -6423,7 +6423,7 @@
         <v>68</v>
       </c>
       <c r="E341">
-        <v>37.38317757009346</v>
+        <v>31.77570093457944</v>
       </c>
     </row>
     <row r="342" spans="1:5">
@@ -6440,7 +6440,7 @@
         <v>69</v>
       </c>
       <c r="E342">
-        <v>35.18518518518519</v>
+        <v>25.92592592592593</v>
       </c>
     </row>
     <row r="343" spans="1:5">
@@ -6457,7 +6457,7 @@
         <v>70</v>
       </c>
       <c r="E343">
-        <v>100</v>
+        <v>47.70642201834863</v>
       </c>
     </row>
     <row r="344" spans="1:5">
@@ -6474,7 +6474,7 @@
         <v>71</v>
       </c>
       <c r="E344">
-        <v>69.56521739130434</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="345" spans="1:5">
@@ -6491,7 +6491,7 @@
         <v>72</v>
       </c>
       <c r="E345">
-        <v>60.37735849056604</v>
+        <v>29.62962962962963</v>
       </c>
     </row>
     <row r="346" spans="1:5">
@@ -6508,7 +6508,7 @@
         <v>73</v>
       </c>
       <c r="E346">
-        <v>68.08510638297872</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="347" spans="1:5">
@@ -6525,7 +6525,7 @@
         <v>74</v>
       </c>
       <c r="E347">
-        <v>68.08510638297872</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="348" spans="1:5">
@@ -6542,7 +6542,7 @@
         <v>75</v>
       </c>
       <c r="E348">
-        <v>66.66666666666666</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="349" spans="1:5">
@@ -6559,7 +6559,7 @@
         <v>76</v>
       </c>
       <c r="E349">
-        <v>65.30612244897959</v>
+        <v>28.84615384615384</v>
       </c>
     </row>
     <row r="350" spans="1:5">
@@ -6576,7 +6576,7 @@
         <v>77</v>
       </c>
       <c r="E350">
-        <v>71.11111111111111</v>
+        <v>26</v>
       </c>
     </row>
     <row r="351" spans="1:5">
@@ -6593,7 +6593,7 @@
         <v>78</v>
       </c>
       <c r="E351">
-        <v>65.30612244897959</v>
+        <v>25</v>
       </c>
     </row>
     <row r="352" spans="1:5">
@@ -6610,7 +6610,7 @@
         <v>79</v>
       </c>
       <c r="E352">
-        <v>61.53846153846154</v>
+        <v>24.29906542056075</v>
       </c>
     </row>
     <row r="353" spans="1:5">
@@ -6627,7 +6627,7 @@
         <v>80</v>
       </c>
       <c r="E353">
-        <v>64</v>
+        <v>24.76190476190476</v>
       </c>
     </row>
     <row r="354" spans="1:5">
@@ -6644,7 +6644,7 @@
         <v>81</v>
       </c>
       <c r="E354">
-        <v>68.08510638297872</v>
+        <v>27.45098039215686</v>
       </c>
     </row>
     <row r="355" spans="1:5">
@@ -6661,7 +6661,7 @@
         <v>82</v>
       </c>
       <c r="E355">
-        <v>60.37735849056604</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="356" spans="1:5">
@@ -6678,7 +6678,7 @@
         <v>83</v>
       </c>
       <c r="E356">
-        <v>61.53846153846154</v>
+        <v>29.90654205607477</v>
       </c>
     </row>
     <row r="357" spans="1:5">
@@ -6695,7 +6695,7 @@
         <v>84</v>
       </c>
       <c r="E357">
-        <v>68.08510638297872</v>
+        <v>25.49019607843137</v>
       </c>
     </row>
     <row r="358" spans="1:5">
@@ -6712,7 +6712,7 @@
         <v>70</v>
       </c>
       <c r="E358">
-        <v>100</v>
+        <v>47.70642201834863</v>
       </c>
     </row>
     <row r="359" spans="1:5">
@@ -6729,7 +6729,7 @@
         <v>65</v>
       </c>
       <c r="E359">
-        <v>35.64356435643565</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="360" spans="1:5">
@@ -6746,7 +6746,7 @@
         <v>66</v>
       </c>
       <c r="E360">
-        <v>35.05154639175258</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="361" spans="1:5">
@@ -6763,7 +6763,7 @@
         <v>67</v>
       </c>
       <c r="E361">
-        <v>31.68316831683168</v>
+        <v>27.72277227722773</v>
       </c>
     </row>
     <row r="362" spans="1:5">
@@ -6780,7 +6780,7 @@
         <v>68</v>
       </c>
       <c r="E362">
-        <v>36.36363636363637</v>
+        <v>32.32323232323232</v>
       </c>
     </row>
     <row r="363" spans="1:5">
@@ -6797,7 +6797,7 @@
         <v>69</v>
       </c>
       <c r="E363">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="364" spans="1:5">
@@ -6814,7 +6814,7 @@
         <v>70</v>
       </c>
       <c r="E364">
-        <v>59.25925925925926</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="365" spans="1:5">
@@ -6831,7 +6831,7 @@
         <v>71</v>
       </c>
       <c r="E365">
-        <v>100</v>
+        <v>38.70967741935484</v>
       </c>
     </row>
     <row r="366" spans="1:5">
@@ -6848,7 +6848,7 @@
         <v>72</v>
       </c>
       <c r="E366">
-        <v>60.37735849056604</v>
+        <v>26</v>
       </c>
     </row>
     <row r="367" spans="1:5">
@@ -6865,7 +6865,7 @@
         <v>73</v>
       </c>
       <c r="E367">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="368" spans="1:5">
@@ -6882,7 +6882,7 @@
         <v>74</v>
       </c>
       <c r="E368">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="369" spans="1:5">
@@ -6899,7 +6899,7 @@
         <v>75</v>
       </c>
       <c r="E369">
-        <v>66.66666666666666</v>
+        <v>27.36842105263158</v>
       </c>
     </row>
     <row r="370" spans="1:5">
@@ -6916,7 +6916,7 @@
         <v>76</v>
       </c>
       <c r="E370">
-        <v>65.30612244897959</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="371" spans="1:5">
@@ -6933,7 +6933,7 @@
         <v>77</v>
       </c>
       <c r="E371">
-        <v>71.11111111111111</v>
+        <v>28.26086956521739</v>
       </c>
     </row>
     <row r="372" spans="1:5">
@@ -6950,7 +6950,7 @@
         <v>78</v>
       </c>
       <c r="E372">
-        <v>65.30612244897959</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="373" spans="1:5">
@@ -6967,7 +6967,7 @@
         <v>79</v>
       </c>
       <c r="E373">
-        <v>61.53846153846154</v>
+        <v>26.26262626262627</v>
       </c>
     </row>
     <row r="374" spans="1:5">
@@ -6984,7 +6984,7 @@
         <v>80</v>
       </c>
       <c r="E374">
-        <v>64</v>
+        <v>26.80412371134021</v>
       </c>
     </row>
     <row r="375" spans="1:5">
@@ -7001,7 +7001,7 @@
         <v>81</v>
       </c>
       <c r="E375">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="376" spans="1:5">
@@ -7018,7 +7018,7 @@
         <v>82</v>
       </c>
       <c r="E376">
-        <v>60.37735849056604</v>
+        <v>26</v>
       </c>
     </row>
     <row r="377" spans="1:5">
@@ -7035,7 +7035,7 @@
         <v>83</v>
       </c>
       <c r="E377">
-        <v>61.53846153846154</v>
+        <v>26.26262626262627</v>
       </c>
     </row>
     <row r="378" spans="1:5">
@@ -7052,7 +7052,7 @@
         <v>84</v>
       </c>
       <c r="E378">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="379" spans="1:5">
@@ -7069,7 +7069,7 @@
         <v>71</v>
       </c>
       <c r="E379">
-        <v>100</v>
+        <v>38.70967741935484</v>
       </c>
     </row>
     <row r="380" spans="1:5">
@@ -7086,7 +7086,7 @@
         <v>65</v>
       </c>
       <c r="E380">
-        <v>33.33333333333333</v>
+        <v>29.62962962962963</v>
       </c>
     </row>
     <row r="381" spans="1:5">
@@ -7103,7 +7103,7 @@
         <v>66</v>
       </c>
       <c r="E381">
-        <v>36.53846153846154</v>
+        <v>32.69230769230769</v>
       </c>
     </row>
     <row r="382" spans="1:5">
@@ -7137,7 +7137,7 @@
         <v>68</v>
       </c>
       <c r="E383">
-        <v>37.73584905660378</v>
+        <v>35.84905660377359</v>
       </c>
     </row>
     <row r="384" spans="1:5">
@@ -7154,7 +7154,7 @@
         <v>69</v>
       </c>
       <c r="E384">
-        <v>35.51401869158879</v>
+        <v>29.90654205607477</v>
       </c>
     </row>
     <row r="385" spans="1:5">
@@ -7171,7 +7171,7 @@
         <v>70</v>
       </c>
       <c r="E385">
-        <v>59.25925925925926</v>
+        <v>31.48148148148148</v>
       </c>
     </row>
     <row r="386" spans="1:5">
@@ -7188,7 +7188,7 @@
         <v>71</v>
       </c>
       <c r="E386">
-        <v>69.56521739130434</v>
+        <v>28</v>
       </c>
     </row>
     <row r="387" spans="1:5">
@@ -7205,7 +7205,7 @@
         <v>72</v>
       </c>
       <c r="E387">
-        <v>100</v>
+        <v>46.72897196261682</v>
       </c>
     </row>
     <row r="388" spans="1:5">
@@ -7222,7 +7222,7 @@
         <v>73</v>
       </c>
       <c r="E388">
-        <v>68.08510638297872</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="389" spans="1:5">
@@ -7239,7 +7239,7 @@
         <v>74</v>
       </c>
       <c r="E389">
-        <v>68.08510638297872</v>
+        <v>29.70297029702971</v>
       </c>
     </row>
     <row r="390" spans="1:5">
@@ -7256,7 +7256,7 @@
         <v>75</v>
       </c>
       <c r="E390">
-        <v>66.66666666666666</v>
+        <v>31.37254901960784</v>
       </c>
     </row>
     <row r="391" spans="1:5">
@@ -7273,7 +7273,7 @@
         <v>76</v>
       </c>
       <c r="E391">
-        <v>65.30612244897959</v>
+        <v>31.06796116504854</v>
       </c>
     </row>
     <row r="392" spans="1:5">
@@ -7290,7 +7290,7 @@
         <v>77</v>
       </c>
       <c r="E392">
-        <v>71.11111111111111</v>
+        <v>28.28282828282829</v>
       </c>
     </row>
     <row r="393" spans="1:5">
@@ -7307,7 +7307,7 @@
         <v>78</v>
       </c>
       <c r="E393">
-        <v>65.30612244897959</v>
+        <v>27.18446601941747</v>
       </c>
     </row>
     <row r="394" spans="1:5">
@@ -7324,7 +7324,7 @@
         <v>79</v>
       </c>
       <c r="E394">
-        <v>61.53846153846154</v>
+        <v>28.30188679245283</v>
       </c>
     </row>
     <row r="395" spans="1:5">
@@ -7341,7 +7341,7 @@
         <v>80</v>
       </c>
       <c r="E395">
-        <v>64</v>
+        <v>26.92307692307693</v>
       </c>
     </row>
     <row r="396" spans="1:5">
@@ -7358,7 +7358,7 @@
         <v>81</v>
       </c>
       <c r="E396">
-        <v>68.08510638297872</v>
+        <v>31.68316831683168</v>
       </c>
     </row>
     <row r="397" spans="1:5">
@@ -7375,7 +7375,7 @@
         <v>82</v>
       </c>
       <c r="E397">
-        <v>60.37735849056604</v>
+        <v>29.90654205607477</v>
       </c>
     </row>
     <row r="398" spans="1:5">
@@ -7392,7 +7392,7 @@
         <v>83</v>
       </c>
       <c r="E398">
-        <v>61.53846153846154</v>
+        <v>32.07547169811321</v>
       </c>
     </row>
     <row r="399" spans="1:5">
@@ -7409,7 +7409,7 @@
         <v>84</v>
       </c>
       <c r="E399">
-        <v>68.08510638297872</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="400" spans="1:5">
@@ -7426,7 +7426,7 @@
         <v>72</v>
       </c>
       <c r="E400">
-        <v>100</v>
+        <v>46.72897196261682</v>
       </c>
     </row>
     <row r="401" spans="1:5">
@@ -7443,7 +7443,7 @@
         <v>65</v>
       </c>
       <c r="E401">
-        <v>35.64356435643565</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="402" spans="1:5">
@@ -7460,7 +7460,7 @@
         <v>66</v>
       </c>
       <c r="E402">
-        <v>35.05154639175258</v>
+        <v>28.8659793814433</v>
       </c>
     </row>
     <row r="403" spans="1:5">
@@ -7477,7 +7477,7 @@
         <v>67</v>
       </c>
       <c r="E403">
-        <v>31.68316831683168</v>
+        <v>27.72277227722773</v>
       </c>
     </row>
     <row r="404" spans="1:5">
@@ -7494,7 +7494,7 @@
         <v>68</v>
       </c>
       <c r="E404">
-        <v>36.36363636363637</v>
+        <v>32.32323232323232</v>
       </c>
     </row>
     <row r="405" spans="1:5">
@@ -7511,7 +7511,7 @@
         <v>69</v>
       </c>
       <c r="E405">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="406" spans="1:5">
@@ -7528,7 +7528,7 @@
         <v>70</v>
       </c>
       <c r="E406">
-        <v>59.25925925925926</v>
+        <v>25.74257425742574</v>
       </c>
     </row>
     <row r="407" spans="1:5">
@@ -7545,7 +7545,7 @@
         <v>71</v>
       </c>
       <c r="E407">
-        <v>100</v>
+        <v>38.70967741935484</v>
       </c>
     </row>
     <row r="408" spans="1:5">
@@ -7562,7 +7562,7 @@
         <v>72</v>
       </c>
       <c r="E408">
-        <v>60.37735849056604</v>
+        <v>26</v>
       </c>
     </row>
     <row r="409" spans="1:5">
@@ -7579,7 +7579,7 @@
         <v>73</v>
       </c>
       <c r="E409">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="410" spans="1:5">
@@ -7596,7 +7596,7 @@
         <v>74</v>
       </c>
       <c r="E410">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="411" spans="1:5">
@@ -7613,7 +7613,7 @@
         <v>75</v>
       </c>
       <c r="E411">
-        <v>66.66666666666666</v>
+        <v>27.36842105263158</v>
       </c>
     </row>
     <row r="412" spans="1:5">
@@ -7630,7 +7630,7 @@
         <v>76</v>
       </c>
       <c r="E412">
-        <v>65.30612244897959</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="413" spans="1:5">
@@ -7647,7 +7647,7 @@
         <v>77</v>
       </c>
       <c r="E413">
-        <v>71.11111111111111</v>
+        <v>28.26086956521739</v>
       </c>
     </row>
     <row r="414" spans="1:5">
@@ -7664,7 +7664,7 @@
         <v>78</v>
       </c>
       <c r="E414">
-        <v>65.30612244897959</v>
+        <v>27.08333333333334</v>
       </c>
     </row>
     <row r="415" spans="1:5">
@@ -7681,7 +7681,7 @@
         <v>79</v>
       </c>
       <c r="E415">
-        <v>61.53846153846154</v>
+        <v>26.26262626262627</v>
       </c>
     </row>
     <row r="416" spans="1:5">
@@ -7698,7 +7698,7 @@
         <v>80</v>
       </c>
       <c r="E416">
-        <v>64</v>
+        <v>26.80412371134021</v>
       </c>
     </row>
     <row r="417" spans="1:5">
@@ -7715,7 +7715,7 @@
         <v>81</v>
       </c>
       <c r="E417">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="418" spans="1:5">
@@ -7732,7 +7732,7 @@
         <v>82</v>
       </c>
       <c r="E418">
-        <v>60.37735849056604</v>
+        <v>26</v>
       </c>
     </row>
     <row r="419" spans="1:5">
@@ -7749,7 +7749,7 @@
         <v>83</v>
       </c>
       <c r="E419">
-        <v>61.53846153846154</v>
+        <v>26.26262626262627</v>
       </c>
     </row>
     <row r="420" spans="1:5">
@@ -7766,7 +7766,7 @@
         <v>84</v>
       </c>
       <c r="E420">
-        <v>68.08510638297872</v>
+        <v>27.6595744680851</v>
       </c>
     </row>
     <row r="421" spans="1:5">
@@ -7783,7 +7783,7 @@
         <v>71</v>
       </c>
       <c r="E421">
-        <v>100</v>
+        <v>38.70967741935484</v>
       </c>
     </row>
   </sheetData>

</xml_diff>